<commit_message>
split the protein level into contrasts, classify and associate, and give every biopsy its own phenotype
</commit_message>
<xml_diff>
--- a/02_Differential_Expression/01_Design/c_data/01_design.xlsx
+++ b/02_Differential_Expression/01_Design/c_data/01_design.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="134">
   <si>
     <t>sheet</t>
   </si>
@@ -194,147 +194,111 @@
     <t>1.2.1</t>
   </si>
   <si>
-    <t>evaluate</t>
+    <t>farver</t>
+  </si>
+  <si>
+    <t>2.1.2</t>
+  </si>
+  <si>
+    <t>fs</t>
+  </si>
+  <si>
+    <t>2.1.0</t>
+  </si>
+  <si>
+    <t>generics</t>
+  </si>
+  <si>
+    <t>0.1.4</t>
+  </si>
+  <si>
+    <t>ggplot2</t>
+  </si>
+  <si>
+    <t>4.0.3</t>
+  </si>
+  <si>
+    <t>ggplotify</t>
+  </si>
+  <si>
+    <t>0.1.3</t>
+  </si>
+  <si>
+    <t>ggrepel</t>
+  </si>
+  <si>
+    <t>0.9.8</t>
+  </si>
+  <si>
+    <t>glue</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>gridGraphics</t>
+  </si>
+  <si>
+    <t>0.5-1</t>
+  </si>
+  <si>
+    <t>gtable</t>
+  </si>
+  <si>
+    <t>0.3.6</t>
+  </si>
+  <si>
+    <t>here</t>
+  </si>
+  <si>
+    <t>1.0.2</t>
+  </si>
+  <si>
+    <t>lifecycle</t>
   </si>
   <si>
     <t>1.0.5</t>
   </si>
   <si>
-    <t>farver</t>
-  </si>
-  <si>
-    <t>2.1.2</t>
-  </si>
-  <si>
-    <t>fastmap</t>
-  </si>
-  <si>
-    <t>1.2.0</t>
-  </si>
-  <si>
-    <t>fs</t>
-  </si>
-  <si>
-    <t>2.1.0</t>
-  </si>
-  <si>
-    <t>generics</t>
-  </si>
-  <si>
-    <t>0.1.4</t>
-  </si>
-  <si>
-    <t>ggplot2</t>
-  </si>
-  <si>
-    <t>4.0.3</t>
-  </si>
-  <si>
-    <t>ggplotify</t>
-  </si>
-  <si>
-    <t>0.1.3</t>
-  </si>
-  <si>
-    <t>ggrepel</t>
-  </si>
-  <si>
-    <t>0.9.8</t>
-  </si>
-  <si>
-    <t>glue</t>
-  </si>
-  <si>
-    <t>1.8.1</t>
-  </si>
-  <si>
-    <t>gridGraphics</t>
-  </si>
-  <si>
-    <t>0.5-1</t>
-  </si>
-  <si>
-    <t>gtable</t>
-  </si>
-  <si>
-    <t>0.3.6</t>
-  </si>
-  <si>
-    <t>here</t>
-  </si>
-  <si>
-    <t>1.0.2</t>
-  </si>
-  <si>
-    <t>htmltools</t>
-  </si>
-  <si>
-    <t>0.5.9</t>
-  </si>
-  <si>
-    <t>htmlwidgets</t>
-  </si>
-  <si>
-    <t>1.6.4</t>
-  </si>
-  <si>
-    <t>jsonlite</t>
+    <t>limma</t>
+  </si>
+  <si>
+    <t>3.68.1</t>
+  </si>
+  <si>
+    <t>Bioconductor 3.23 (R 4.6.0)</t>
+  </si>
+  <si>
+    <t>magrittr</t>
+  </si>
+  <si>
+    <t>2.0.5</t>
+  </si>
+  <si>
+    <t>pillar</t>
+  </si>
+  <si>
+    <t>1.11.1</t>
+  </si>
+  <si>
+    <t>pkgconfig</t>
+  </si>
+  <si>
+    <t>2.0.3</t>
+  </si>
+  <si>
+    <t>Polychrome</t>
+  </si>
+  <si>
+    <t>1.5.4</t>
+  </si>
+  <si>
+    <t>proteoDA</t>
   </si>
   <si>
     <t>2.0.0</t>
   </si>
   <si>
-    <t>knitr</t>
-  </si>
-  <si>
-    <t>1.51</t>
-  </si>
-  <si>
-    <t>lifecycle</t>
-  </si>
-  <si>
-    <t>limma</t>
-  </si>
-  <si>
-    <t>3.68.1</t>
-  </si>
-  <si>
-    <t>Bioconductor 3.23 (R 4.6.0)</t>
-  </si>
-  <si>
-    <t>magrittr</t>
-  </si>
-  <si>
-    <t>2.0.5</t>
-  </si>
-  <si>
-    <t>otel</t>
-  </si>
-  <si>
-    <t>0.2.0</t>
-  </si>
-  <si>
-    <t>pillar</t>
-  </si>
-  <si>
-    <t>1.11.1</t>
-  </si>
-  <si>
-    <t>pkgconfig</t>
-  </si>
-  <si>
-    <t>2.0.3</t>
-  </si>
-  <si>
-    <t>Polychrome</t>
-  </si>
-  <si>
-    <t>1.5.4</t>
-  </si>
-  <si>
-    <t>proteoDA</t>
-  </si>
-  <si>
     <t>Github (ByrumLab/proteoDA@ba99c77b8d401ef2e3ed95a9c0881ef19feab938)</t>
   </si>
   <si>
@@ -377,12 +341,6 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
-    <t>rmarkdown</t>
-  </si>
-  <si>
-    <t>2.31</t>
-  </si>
-  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -450,12 +408,6 @@
   </si>
   <si>
     <t>2.0.1</t>
-  </si>
-  <si>
-    <t>xfun</t>
-  </si>
-  <si>
-    <t>0.57</t>
   </si>
   <si>
     <t>yaml</t>
@@ -1038,7 +990,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1236,15 +1188,15 @@
         <v>81</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
         <v>49</v>
@@ -1252,10 +1204,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
         <v>49</v>
@@ -1263,10 +1215,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C21" t="s">
         <v>49</v>
@@ -1274,10 +1226,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
         <v>49</v>
@@ -1285,32 +1237,32 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C25" t="s">
         <v>49</v>
@@ -1318,10 +1270,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
         <v>49</v>
@@ -1329,10 +1281,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
         <v>49</v>
@@ -1340,10 +1292,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
         <v>49</v>
@@ -1351,32 +1303,32 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B31" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
         <v>49</v>
@@ -1384,10 +1336,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C32" t="s">
         <v>49</v>
@@ -1395,10 +1347,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B33" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C33" t="s">
         <v>49</v>
@@ -1406,10 +1358,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C34" t="s">
         <v>49</v>
@@ -1417,10 +1369,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B35" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C35" t="s">
         <v>49</v>
@@ -1428,21 +1380,21 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B37" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
@@ -1450,10 +1402,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B38" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
@@ -1461,10 +1413,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B39" t="s">
-        <v>124</v>
+        <v>57</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
@@ -1472,10 +1424,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B40" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
@@ -1483,21 +1435,21 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B41" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C41" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B42" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -1505,111 +1457,12 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B43" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>133</v>
-      </c>
-      <c r="B44" t="s">
-        <v>134</v>
-      </c>
-      <c r="C44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>135</v>
-      </c>
-      <c r="B45" t="s">
-        <v>136</v>
-      </c>
-      <c r="C45" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>137</v>
-      </c>
-      <c r="B46" t="s">
-        <v>138</v>
-      </c>
-      <c r="C46" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>139</v>
-      </c>
-      <c r="B47" t="s">
-        <v>57</v>
-      </c>
-      <c r="C47" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" t="s">
-        <v>140</v>
-      </c>
-      <c r="B48" t="s">
-        <v>141</v>
-      </c>
-      <c r="C48" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>142</v>
-      </c>
-      <c r="B49" t="s">
-        <v>143</v>
-      </c>
-      <c r="C49" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
-        <v>144</v>
-      </c>
-      <c r="B50" t="s">
-        <v>145</v>
-      </c>
-      <c r="C50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
-        <v>146</v>
-      </c>
-      <c r="B51" t="s">
-        <v>147</v>
-      </c>
-      <c r="C51" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>148</v>
-      </c>
-      <c r="B52" t="s">
-        <v>149</v>
-      </c>
-      <c r="C52" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerun every step on limpa; the lists and the panel now sit at their chance lines
</commit_message>
<xml_diff>
--- a/02_Differential_Expression/01_Design/c_data/01_design.xlsx
+++ b/02_Differential_Expression/01_Design/c_data/01_design.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
   <si>
     <t>sheet</t>
   </si>
@@ -35,7 +35,7 @@
     <t>correlation_strata</t>
   </si>
   <si>
-    <t>Within-subject correlation from duplicateCorrelation, blocked by subject.</t>
+    <t>Within-subject correlation from limpa's fit, blocked by subject.</t>
   </si>
   <si>
     <t>input_manifest</t>
@@ -131,7 +131,7 @@
     <t>correlation</t>
   </si>
   <si>
-    <t>within subject, subject random (unweighted matrix correlation)</t>
+    <t>within subject, from limpa's dpcDE fit with subject blocked</t>
   </si>
   <si>
     <t>input</t>
@@ -143,13 +143,13 @@
     <t>md5</t>
   </si>
   <si>
-    <t>normalized</t>
-  </si>
-  <si>
-    <t>01_Preprocess/02_Normalization/c_data/DAList_normalized.rds</t>
-  </si>
-  <si>
-    <t>3759b18a8f3aa42799daa3bda21b03fa</t>
+    <t>proteins</t>
+  </si>
+  <si>
+    <t>01_Preprocess/03_Quantification/c_data/proteins.rds</t>
+  </si>
+  <si>
+    <t>34ef12f3ddbea70e6840925bab8692c5</t>
   </si>
   <si>
     <t>package</t>
@@ -176,16 +176,10 @@
     <t>3.6.6</t>
   </si>
   <si>
-    <t>colorspace</t>
-  </si>
-  <si>
-    <t>2.1-2</t>
-  </si>
-  <si>
-    <t>digest</t>
-  </si>
-  <si>
-    <t>0.6.39</t>
+    <t>data.table</t>
+  </si>
+  <si>
+    <t>1.18.4</t>
   </si>
   <si>
     <t>dplyr</t>
@@ -194,60 +188,18 @@
     <t>1.2.1</t>
   </si>
   <si>
-    <t>farver</t>
-  </si>
-  <si>
-    <t>2.1.2</t>
-  </si>
-  <si>
-    <t>fs</t>
-  </si>
-  <si>
-    <t>2.1.0</t>
-  </si>
-  <si>
     <t>generics</t>
   </si>
   <si>
     <t>0.1.4</t>
   </si>
   <si>
-    <t>ggplot2</t>
-  </si>
-  <si>
-    <t>4.0.3</t>
-  </si>
-  <si>
-    <t>ggplotify</t>
-  </si>
-  <si>
-    <t>0.1.3</t>
-  </si>
-  <si>
-    <t>ggrepel</t>
-  </si>
-  <si>
-    <t>0.9.8</t>
-  </si>
-  <si>
     <t>glue</t>
   </si>
   <si>
     <t>1.8.1</t>
   </si>
   <si>
-    <t>gridGraphics</t>
-  </si>
-  <si>
-    <t>0.5-1</t>
-  </si>
-  <si>
-    <t>gtable</t>
-  </si>
-  <si>
-    <t>0.3.6</t>
-  </si>
-  <si>
     <t>here</t>
   </si>
   <si>
@@ -269,6 +221,12 @@
     <t>Bioconductor 3.23 (R 4.6.0)</t>
   </si>
   <si>
+    <t>limpa</t>
+  </si>
+  <si>
+    <t>1.4.2</t>
+  </si>
+  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -287,45 +245,12 @@
     <t>2.0.3</t>
   </si>
   <si>
-    <t>Polychrome</t>
-  </si>
-  <si>
-    <t>1.5.4</t>
-  </si>
-  <si>
-    <t>proteoDA</t>
-  </si>
-  <si>
-    <t>2.0.0</t>
-  </si>
-  <si>
-    <t>Github (ByrumLab/proteoDA@ba99c77b8d401ef2e3ed95a9c0881ef19feab938)</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
     <t>2.6.1</t>
   </si>
   <si>
-    <t>rappdirs</t>
-  </si>
-  <si>
-    <t>0.3.4</t>
-  </si>
-  <si>
-    <t>RColorBrewer</t>
-  </si>
-  <si>
-    <t>1.1-3</t>
-  </si>
-  <si>
-    <t>Rcpp</t>
-  </si>
-  <si>
-    <t>1.1.1-1.1</t>
-  </si>
-  <si>
     <t>renv</t>
   </si>
   <si>
@@ -347,24 +272,6 @@
     <t>2.1.1</t>
   </si>
   <si>
-    <t>S7</t>
-  </si>
-  <si>
-    <t>0.2.2</t>
-  </si>
-  <si>
-    <t>scales</t>
-  </si>
-  <si>
-    <t>1.4.0</t>
-  </si>
-  <si>
-    <t>scatterplot3d</t>
-  </si>
-  <si>
-    <t>0.3-45</t>
-  </si>
-  <si>
     <t>sessioninfo</t>
   </si>
   <si>
@@ -377,18 +284,6 @@
     <t>1.5.1</t>
   </si>
   <si>
-    <t>stringi</t>
-  </si>
-  <si>
-    <t>1.8.7</t>
-  </si>
-  <si>
-    <t>stringr</t>
-  </si>
-  <si>
-    <t>1.6.0</t>
-  </si>
-  <si>
     <t>tibble</t>
   </si>
   <si>
@@ -408,12 +303,6 @@
   </si>
   <si>
     <t>2.0.1</t>
-  </si>
-  <si>
-    <t>yulab.utils</t>
-  </si>
-  <si>
-    <t>0.2.4</t>
   </si>
 </sst>
 </file>
@@ -942,7 +831,7 @@
         <v>37</v>
       </c>
       <c r="B2">
-        <v>0.18906629970961</v>
+        <v>0.1702823336442219</v>
       </c>
     </row>
   </sheetData>
@@ -984,7 +873,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1094,26 +983,26 @@
         <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s">
         <v>66</v>
-      </c>
-      <c r="B11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
         <v>49</v>
@@ -1121,10 +1010,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
         <v>49</v>
@@ -1132,10 +1021,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
         <v>49</v>
@@ -1143,10 +1032,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
         <v>49</v>
@@ -1154,10 +1043,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
         <v>49</v>
@@ -1165,32 +1054,32 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C19" t="s">
         <v>49</v>
@@ -1198,10 +1087,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
         <v>49</v>
@@ -1209,10 +1098,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
         <v>49</v>
@@ -1220,10 +1109,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
         <v>49</v>
@@ -1237,216 +1126,18 @@
         <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B24" t="s">
         <v>94</v>
       </c>
-      <c r="B24" t="s">
-        <v>95</v>
-      </c>
       <c r="C24" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>96</v>
-      </c>
-      <c r="B25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>98</v>
-      </c>
-      <c r="B26" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>100</v>
-      </c>
-      <c r="B27" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" t="s">
-        <v>103</v>
-      </c>
-      <c r="C28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>104</v>
-      </c>
-      <c r="B29" t="s">
-        <v>105</v>
-      </c>
-      <c r="C29" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>107</v>
-      </c>
-      <c r="B30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C30" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" t="s">
-        <v>110</v>
-      </c>
-      <c r="C31" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>111</v>
-      </c>
-      <c r="B32" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>113</v>
-      </c>
-      <c r="B33" t="s">
-        <v>114</v>
-      </c>
-      <c r="C33" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>117</v>
-      </c>
-      <c r="B35" t="s">
-        <v>118</v>
-      </c>
-      <c r="C35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>119</v>
-      </c>
-      <c r="B36" t="s">
-        <v>120</v>
-      </c>
-      <c r="C36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>121</v>
-      </c>
-      <c r="B37" t="s">
-        <v>122</v>
-      </c>
-      <c r="C37" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>123</v>
-      </c>
-      <c r="B38" t="s">
-        <v>124</v>
-      </c>
-      <c r="C38" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>125</v>
-      </c>
-      <c r="B39" t="s">
-        <v>57</v>
-      </c>
-      <c r="C39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>126</v>
-      </c>
-      <c r="B40" t="s">
-        <v>127</v>
-      </c>
-      <c r="C40" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>128</v>
-      </c>
-      <c r="B41" t="s">
-        <v>129</v>
-      </c>
-      <c r="C41" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>130</v>
-      </c>
-      <c r="B42" t="s">
-        <v>131</v>
-      </c>
-      <c r="C42" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
every script writes its workbook through write_workbook, and proteoDA stops leaving Rplots.pdf around
</commit_message>
<xml_diff>
--- a/02_Differential_Expression/01_Design/c_data/01_design.xlsx
+++ b/02_Differential_Expression/01_Design/c_data/01_design.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="146">
   <si>
     <t>sheet</t>
   </si>
@@ -161,6 +161,15 @@
     <t>source</t>
   </si>
   <si>
+    <t>BiocGenerics</t>
+  </si>
+  <si>
+    <t>0.58.0</t>
+  </si>
+  <si>
+    <t>Bioconductor 3.23 (R 4.6.0)</t>
+  </si>
+  <si>
     <t>BiocManager</t>
   </si>
   <si>
@@ -170,42 +179,141 @@
     <t>CRAN (R 4.6.0)</t>
   </si>
   <si>
+    <t>circlize</t>
+  </si>
+  <si>
+    <t>0.4.18</t>
+  </si>
+  <si>
     <t>cli</t>
   </si>
   <si>
     <t>3.6.6</t>
   </si>
   <si>
+    <t>clue</t>
+  </si>
+  <si>
+    <t>0.3-68</t>
+  </si>
+  <si>
+    <t>cluster</t>
+  </si>
+  <si>
+    <t>2.1.8.2</t>
+  </si>
+  <si>
+    <t>codetools</t>
+  </si>
+  <si>
+    <t>0.2-20</t>
+  </si>
+  <si>
+    <t>colorspace</t>
+  </si>
+  <si>
+    <t>2.1-2</t>
+  </si>
+  <si>
+    <t>ComplexHeatmap</t>
+  </si>
+  <si>
+    <t>2.28.0</t>
+  </si>
+  <si>
+    <t>crayon</t>
+  </si>
+  <si>
+    <t>1.5.3</t>
+  </si>
+  <si>
     <t>data.table</t>
   </si>
   <si>
     <t>1.18.4</t>
   </si>
   <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>0.6.39</t>
+  </si>
+  <si>
+    <t>doParallel</t>
+  </si>
+  <si>
+    <t>1.0.17</t>
+  </si>
+  <si>
     <t>dplyr</t>
   </si>
   <si>
     <t>1.2.1</t>
   </si>
   <si>
+    <t>farver</t>
+  </si>
+  <si>
+    <t>2.1.2</t>
+  </si>
+  <si>
+    <t>foreach</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
     <t>generics</t>
   </si>
   <si>
     <t>0.1.4</t>
   </si>
   <si>
+    <t>GetoptLong</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
+    <t>ggplot2</t>
+  </si>
+  <si>
+    <t>4.0.3</t>
+  </si>
+  <si>
+    <t>GlobalOptions</t>
+  </si>
+  <si>
     <t>glue</t>
   </si>
   <si>
     <t>1.8.1</t>
   </si>
   <si>
+    <t>gtable</t>
+  </si>
+  <si>
+    <t>0.3.6</t>
+  </si>
+  <si>
     <t>here</t>
   </si>
   <si>
     <t>1.0.2</t>
   </si>
   <si>
+    <t>IRanges</t>
+  </si>
+  <si>
+    <t>2.46.0</t>
+  </si>
+  <si>
+    <t>iterators</t>
+  </si>
+  <si>
+    <t>1.0.14</t>
+  </si>
+  <si>
     <t>lifecycle</t>
   </si>
   <si>
@@ -218,9 +326,6 @@
     <t>3.68.1</t>
   </si>
   <si>
-    <t>Bioconductor 3.23 (R 4.6.0)</t>
-  </si>
-  <si>
     <t>limpa</t>
   </si>
   <si>
@@ -233,6 +338,12 @@
     <t>2.0.5</t>
   </si>
   <si>
+    <t>matrixStats</t>
+  </si>
+  <si>
+    <t>1.5.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -245,18 +356,36 @@
     <t>2.0.3</t>
   </si>
   <si>
+    <t>png</t>
+  </si>
+  <si>
+    <t>0.1-9</t>
+  </si>
+  <si>
     <t>R6</t>
   </si>
   <si>
     <t>2.6.1</t>
   </si>
   <si>
+    <t>RColorBrewer</t>
+  </si>
+  <si>
+    <t>1.1-3</t>
+  </si>
+  <si>
     <t>renv</t>
   </si>
   <si>
     <t>1.2.3</t>
   </si>
   <si>
+    <t>rjson</t>
+  </si>
+  <si>
+    <t>0.2.23</t>
+  </si>
+  <si>
     <t>rlang</t>
   </si>
   <si>
@@ -272,10 +401,34 @@
     <t>2.1.1</t>
   </si>
   <si>
+    <t>S4Vectors</t>
+  </si>
+  <si>
+    <t>0.50.0</t>
+  </si>
+  <si>
+    <t>S7</t>
+  </si>
+  <si>
+    <t>0.2.2</t>
+  </si>
+  <si>
+    <t>scales</t>
+  </si>
+  <si>
+    <t>1.4.0</t>
+  </si>
+  <si>
     <t>sessioninfo</t>
   </si>
   <si>
     <t>1.2.4</t>
+  </si>
+  <si>
+    <t>shape</t>
+  </si>
+  <si>
+    <t>1.4.6.1</t>
   </si>
   <si>
     <t>statmod</t>
@@ -873,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -906,84 +1059,84 @@
         <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -994,7 +1147,7 @@
         <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1005,7 +1158,7 @@
         <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1016,7 +1169,7 @@
         <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1027,7 +1180,7 @@
         <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1038,7 +1191,7 @@
         <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1049,7 +1202,7 @@
         <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1060,84 +1213,370 @@
         <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s">
         <v>82</v>
       </c>
-      <c r="B18" t="s">
-        <v>83</v>
-      </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" t="s">
         <v>84</v>
       </c>
-      <c r="B19" t="s">
-        <v>85</v>
-      </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" t="s">
         <v>86</v>
       </c>
-      <c r="B20" t="s">
-        <v>87</v>
-      </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" t="s">
         <v>91</v>
       </c>
-      <c r="B23" t="s">
-        <v>92</v>
-      </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
         <v>93</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
         <v>94</v>
       </c>
-      <c r="C24" t="s">
-        <v>81</v>
+      <c r="B25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>100</v>
+      </c>
+      <c r="B28" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" t="s">
+        <v>105</v>
+      </c>
+      <c r="C30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" t="s">
+        <v>119</v>
+      </c>
+      <c r="C37" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B38" t="s">
+        <v>121</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>125</v>
+      </c>
+      <c r="B40" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>129</v>
+      </c>
+      <c r="B42" t="s">
+        <v>130</v>
+      </c>
+      <c r="C42" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>131</v>
+      </c>
+      <c r="B43" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>133</v>
+      </c>
+      <c r="B44" t="s">
+        <v>134</v>
+      </c>
+      <c r="C44" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>135</v>
+      </c>
+      <c r="B45" t="s">
+        <v>136</v>
+      </c>
+      <c r="C45" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" t="s">
+        <v>138</v>
+      </c>
+      <c r="C46" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>139</v>
+      </c>
+      <c r="B47" t="s">
+        <v>140</v>
+      </c>
+      <c r="C47" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>141</v>
+      </c>
+      <c r="B48" t="s">
+        <v>76</v>
+      </c>
+      <c r="C48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>142</v>
+      </c>
+      <c r="B49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>144</v>
+      </c>
+      <c r="B50" t="s">
+        <v>145</v>
+      </c>
+      <c r="C50" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>